<commit_message>
eval: bulk up corpus (23-row tables, 20-run logs, dense annotated diagrams)
</commit_message>
<xml_diff>
--- a/eval/dataset/files/components.xlsx
+++ b/eval/dataset/files/components.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,67 +449,262 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ammeter</t>
+          <t>resistor 100 ohm</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>350</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>voltmeter</t>
+          <t>resistor 150 ohm</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>320</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>rheostat</t>
+          <t>resistor 470 ohm</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>180</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>battery 12V</t>
+          <t>ammeter</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>220</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>voltmeter</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>rheostat 500 ohm</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>battery 12V</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>battery 6V</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>wire red 1m</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>15</v>
+      </c>
+      <c r="C11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>wire black 1m</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>crocodile clips</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>30</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>breadboard</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>bulb 6V</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fuse 1A</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>multimeter</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>screwdriver set</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>lab manual</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>storage tray</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7">
-        <f>SUM(B2:B6)</f>
+      <c r="B22">
+        <f>SUM(B2:B21)</f>
         <v/>
       </c>
-      <c r="C7">
-        <f>SUM(C2:C6)</f>
+      <c r="C22">
+        <f>SUM(C2:C21)</f>
         <v/>
       </c>
     </row>

</xml_diff>